<commit_message>
Ajout de la liaison avec le fichier des capacités
</commit_message>
<xml_diff>
--- a/Data/Survivants-Zombicide.xlsx
+++ b/Data/Survivants-Zombicide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anian\OneDrive\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3BC8350-2FA1-4243-BE65-9B5A159607F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A2FCDAC-0FC7-4498-94FA-49B9308171A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{8F225D54-4EF0-458C-80A6-925776A8C32C}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$1:$M$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="167">
   <si>
     <t>Personnage</t>
   </si>
@@ -424,16 +424,139 @@
   </si>
   <si>
     <t>Zoe</t>
+  </si>
+  <si>
+    <t>Power 1</t>
+  </si>
+  <si>
+    <t>Power 2</t>
+  </si>
+  <si>
+    <t>Power 3</t>
+  </si>
+  <si>
+    <t>Power 4</t>
+  </si>
+  <si>
+    <t>Power 5</t>
+  </si>
+  <si>
+    <t>Power 6</t>
+  </si>
+  <si>
+    <t>Power 7</t>
+  </si>
+  <si>
+    <t>+1 Damage: Magic</t>
+  </si>
+  <si>
+    <t>+1 Action</t>
+  </si>
+  <si>
+    <t>+1 die: Magic</t>
+  </si>
+  <si>
+    <t>Slippery</t>
+  </si>
+  <si>
+    <t>+1 free Combat Action</t>
+  </si>
+  <si>
+    <t>+1 to dice roll: Magic</t>
+  </si>
+  <si>
+    <t>Regeneration</t>
+  </si>
+  <si>
+    <t>Bloodlust: Melee</t>
+  </si>
+  <si>
+    <t>+1 free Magic Action</t>
+  </si>
+  <si>
+    <t>+1 free Melee Action</t>
+  </si>
+  <si>
+    <t>+1 to dice roll: Combat</t>
+  </si>
+  <si>
+    <t>Taunt</t>
+  </si>
+  <si>
+    <t>Frenzy: Combat</t>
+  </si>
+  <si>
+    <t>Barbarian</t>
+  </si>
+  <si>
+    <t>Iron hide</t>
+  </si>
+  <si>
+    <t>Destiny</t>
+  </si>
+  <si>
+    <t>Spellcaster</t>
+  </si>
+  <si>
+    <t>+1 die: Combat</t>
+  </si>
+  <si>
+    <t>Roll 6: +1 die Combat</t>
+  </si>
+  <si>
+    <t>+1 Zone per Move</t>
+  </si>
+  <si>
+    <t>Point-blank</t>
+  </si>
+  <si>
+    <t>Jump</t>
+  </si>
+  <si>
+    <t>+1 free Move Action</t>
+  </si>
+  <si>
+    <t>+1 to dice roll: Ranged</t>
+  </si>
+  <si>
+    <t>+1 free Search Action</t>
+  </si>
+  <si>
+    <t>+1 die: Melee</t>
+  </si>
+  <si>
+    <t>Reaper: Combat</t>
+  </si>
+  <si>
+    <t>+1 to dice roll: Melee</t>
+  </si>
+  <si>
+    <t>Starts with a Curved Dagger</t>
+  </si>
+  <si>
+    <t>+1 Damage: Melee</t>
+  </si>
+  <si>
+    <t>Rotten</t>
+  </si>
+  <si>
+    <t>Born leader</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -459,8 +582,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -775,10 +899,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7E558BA-FFD6-48B0-805B-6B97F54719C5}">
-  <dimension ref="A1:F218"/>
+  <dimension ref="A1:M218"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="13" max="13" width="22.26953125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -797,8 +924,29 @@
       <c r="F1" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G1" t="s">
+        <v>128</v>
+      </c>
+      <c r="H1" t="s">
+        <v>129</v>
+      </c>
+      <c r="I1" t="s">
+        <v>130</v>
+      </c>
+      <c r="J1" t="s">
+        <v>131</v>
+      </c>
+      <c r="K1" t="s">
+        <v>132</v>
+      </c>
+      <c r="L1" t="s">
+        <v>133</v>
+      </c>
+      <c r="M1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -808,8 +956,29 @@
       <c r="C2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G2" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -819,8 +988,29 @@
       <c r="C3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G3" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -830,8 +1020,29 @@
       <c r="C4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G4" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -841,8 +1052,29 @@
       <c r="C5" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G5" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -858,8 +1090,29 @@
       <c r="E6" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G6" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -869,8 +1122,29 @@
       <c r="C7" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G7" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="L7" t="s">
+        <v>149</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -880,8 +1154,29 @@
       <c r="C8" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G8" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -891,8 +1186,29 @@
       <c r="C9" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G9" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -902,8 +1218,29 @@
       <c r="C10" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G10" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -913,8 +1250,11 @@
       <c r="C11" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H11" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -927,8 +1267,11 @@
       <c r="D12" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H12" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -938,8 +1281,11 @@
       <c r="C13" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H13" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -949,8 +1295,11 @@
       <c r="C14" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H14" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -960,8 +1309,11 @@
       <c r="C15" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H15" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -971,8 +1323,11 @@
       <c r="C16" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H16" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -985,8 +1340,11 @@
       <c r="D17" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H17" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>24</v>
       </c>
@@ -996,8 +1354,11 @@
       <c r="C18" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H18" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -1007,8 +1368,11 @@
       <c r="C19" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H19" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>26</v>
       </c>
@@ -1021,8 +1385,11 @@
       <c r="D20" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H20" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>27</v>
       </c>
@@ -1032,8 +1399,11 @@
       <c r="C21" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H21" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>28</v>
       </c>
@@ -1043,8 +1413,11 @@
       <c r="C22" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H22" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>29</v>
       </c>
@@ -1054,8 +1427,11 @@
       <c r="C23" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H23" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>30</v>
       </c>
@@ -1065,8 +1441,11 @@
       <c r="C24" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H24" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>31</v>
       </c>
@@ -1076,8 +1455,11 @@
       <c r="C25" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H25" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>32</v>
       </c>
@@ -1087,8 +1469,11 @@
       <c r="C26" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H26" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>33</v>
       </c>
@@ -1098,8 +1483,11 @@
       <c r="C27" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H27" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>34</v>
       </c>
@@ -1109,8 +1497,11 @@
       <c r="C28" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H28" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>35</v>
       </c>
@@ -1120,8 +1511,11 @@
       <c r="C29" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H29" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>36</v>
       </c>
@@ -1131,8 +1525,11 @@
       <c r="C30" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H30" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>37</v>
       </c>
@@ -1148,8 +1545,11 @@
       <c r="E31" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H31" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>38</v>
       </c>
@@ -1159,8 +1559,11 @@
       <c r="C32" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H32" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>39</v>
       </c>
@@ -1173,8 +1576,11 @@
       <c r="F33" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H33" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>42</v>
       </c>
@@ -1184,8 +1590,11 @@
       <c r="C34" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H34" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>43</v>
       </c>
@@ -1195,8 +1604,11 @@
       <c r="C35" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H35" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>44</v>
       </c>
@@ -1206,8 +1618,11 @@
       <c r="C36" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H36" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>45</v>
       </c>
@@ -1217,8 +1632,11 @@
       <c r="C37" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H37" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>46</v>
       </c>
@@ -1228,8 +1646,11 @@
       <c r="C38" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H38" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>47</v>
       </c>
@@ -1239,8 +1660,11 @@
       <c r="C39" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H39" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>48</v>
       </c>
@@ -1250,8 +1674,11 @@
       <c r="C40" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H40" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>49</v>
       </c>
@@ -1264,8 +1691,11 @@
       <c r="D41" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H41" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>50</v>
       </c>
@@ -1275,8 +1705,11 @@
       <c r="C42" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H42" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>51</v>
       </c>
@@ -1286,8 +1719,11 @@
       <c r="C43" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H43" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>52</v>
       </c>
@@ -1297,8 +1733,11 @@
       <c r="C44" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H44" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>53</v>
       </c>
@@ -1308,8 +1747,11 @@
       <c r="C45" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H45" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>54</v>
       </c>
@@ -1319,8 +1761,11 @@
       <c r="C46" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H46" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>55</v>
       </c>
@@ -1330,8 +1775,11 @@
       <c r="C47" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="H47" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>56</v>
       </c>
@@ -1341,8 +1789,11 @@
       <c r="C48" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H48" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>57</v>
       </c>
@@ -1352,8 +1803,11 @@
       <c r="C49" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H49" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>58</v>
       </c>
@@ -1363,8 +1817,11 @@
       <c r="C50" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H50" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>59</v>
       </c>
@@ -1377,8 +1834,11 @@
       <c r="D51" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H51" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>60</v>
       </c>
@@ -1391,8 +1851,11 @@
       <c r="D52" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H52" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>61</v>
       </c>
@@ -1402,8 +1865,11 @@
       <c r="C53" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H53" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>62</v>
       </c>
@@ -1413,8 +1879,11 @@
       <c r="C54" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H54" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>63</v>
       </c>
@@ -1424,8 +1893,11 @@
       <c r="C55" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H55" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>64</v>
       </c>
@@ -1435,8 +1907,11 @@
       <c r="C56" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H56" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>65</v>
       </c>
@@ -1446,8 +1921,11 @@
       <c r="C57" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H57" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>66</v>
       </c>
@@ -1457,8 +1935,11 @@
       <c r="C58" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H58" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>67</v>
       </c>
@@ -1468,8 +1949,11 @@
       <c r="C59" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H59" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>68</v>
       </c>
@@ -1479,8 +1963,11 @@
       <c r="C60" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H60" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>69</v>
       </c>
@@ -1490,8 +1977,11 @@
       <c r="C61" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H61" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>70</v>
       </c>
@@ -1504,8 +1994,11 @@
       <c r="D62" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H62" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>71</v>
       </c>
@@ -1515,8 +2008,11 @@
       <c r="C63" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H63" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>72</v>
       </c>
@@ -1529,8 +2025,11 @@
       <c r="D64" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H64" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>73</v>
       </c>
@@ -1543,8 +2042,11 @@
       <c r="D65" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H65" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>74</v>
       </c>
@@ -1557,8 +2059,11 @@
       <c r="D66" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H66" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>75</v>
       </c>
@@ -1568,8 +2073,11 @@
       <c r="C67" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H67" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>76</v>
       </c>
@@ -1579,8 +2087,11 @@
       <c r="C68" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H68" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>77</v>
       </c>
@@ -1590,8 +2101,11 @@
       <c r="C69" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H69" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>78</v>
       </c>
@@ -1601,8 +2115,11 @@
       <c r="C70" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H70" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>79</v>
       </c>
@@ -1615,8 +2132,11 @@
       <c r="D71" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H71" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>80</v>
       </c>
@@ -1629,8 +2149,11 @@
       <c r="D72" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H72" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>81</v>
       </c>
@@ -1640,8 +2163,11 @@
       <c r="C73" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H73" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>82</v>
       </c>
@@ -1651,8 +2177,11 @@
       <c r="C74" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H74" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>83</v>
       </c>
@@ -1662,8 +2191,11 @@
       <c r="C75" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H75" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>84</v>
       </c>
@@ -1673,8 +2205,11 @@
       <c r="C76" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H76" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>86</v>
       </c>
@@ -1684,8 +2219,11 @@
       <c r="C77" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H77" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>87</v>
       </c>
@@ -1695,8 +2233,11 @@
       <c r="C78" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H78" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>88</v>
       </c>
@@ -1706,8 +2247,11 @@
       <c r="C79" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H79" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>89</v>
       </c>
@@ -1720,8 +2264,11 @@
       <c r="D80" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H80" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>90</v>
       </c>
@@ -1731,8 +2278,11 @@
       <c r="C81" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H81" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>91</v>
       </c>
@@ -1742,8 +2292,11 @@
       <c r="C82" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H82" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>92</v>
       </c>
@@ -1753,8 +2306,11 @@
       <c r="C83" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H83" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>93</v>
       </c>
@@ -1767,8 +2323,11 @@
       <c r="D84" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H84" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>94</v>
       </c>
@@ -1778,8 +2337,11 @@
       <c r="C85" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H85" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>95</v>
       </c>
@@ -1789,8 +2351,11 @@
       <c r="C86" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H86" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>96</v>
       </c>
@@ -1800,8 +2365,11 @@
       <c r="C87" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H87" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>97</v>
       </c>
@@ -1811,8 +2379,11 @@
       <c r="C88" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H88" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>98</v>
       </c>
@@ -1822,8 +2393,11 @@
       <c r="C89" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H89" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>99</v>
       </c>
@@ -1833,8 +2407,11 @@
       <c r="C90" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H90" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>100</v>
       </c>
@@ -1847,8 +2424,11 @@
       <c r="D91" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H91" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>101</v>
       </c>
@@ -1858,8 +2438,11 @@
       <c r="C92" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H92" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>102</v>
       </c>
@@ -1869,8 +2452,11 @@
       <c r="C93" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H93" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>103</v>
       </c>
@@ -1880,8 +2466,11 @@
       <c r="C94" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H94" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>104</v>
       </c>
@@ -1894,8 +2483,11 @@
       <c r="D95" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H95" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>105</v>
       </c>
@@ -1905,8 +2497,11 @@
       <c r="C96" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H96" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>106</v>
       </c>
@@ -1916,8 +2511,11 @@
       <c r="C97" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H97" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>107</v>
       </c>
@@ -1927,8 +2525,11 @@
       <c r="C98" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H98" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>108</v>
       </c>
@@ -1938,8 +2539,11 @@
       <c r="C99" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H99" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>109</v>
       </c>
@@ -1949,8 +2553,11 @@
       <c r="C100" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H100" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>110</v>
       </c>
@@ -1960,8 +2567,11 @@
       <c r="C101" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H101" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>111</v>
       </c>
@@ -1971,8 +2581,11 @@
       <c r="C102" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H102" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>112</v>
       </c>
@@ -1982,8 +2595,11 @@
       <c r="C103" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H103" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>113</v>
       </c>
@@ -1993,8 +2609,11 @@
       <c r="C104" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H104" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>114</v>
       </c>
@@ -2007,8 +2626,11 @@
       <c r="D105" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H105" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>115</v>
       </c>
@@ -2021,8 +2643,11 @@
       <c r="D106" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H106" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>116</v>
       </c>
@@ -2032,8 +2657,11 @@
       <c r="C107" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H107" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>117</v>
       </c>
@@ -2046,8 +2674,11 @@
       <c r="D108" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H108" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>118</v>
       </c>
@@ -2063,8 +2694,11 @@
       <c r="E109" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H109" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>119</v>
       </c>
@@ -2074,8 +2708,11 @@
       <c r="C110" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H110" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>120</v>
       </c>
@@ -2088,8 +2725,11 @@
       <c r="D111" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="H111" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>121</v>
       </c>
@@ -2102,8 +2742,11 @@
       <c r="D112" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H112" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="113" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>122</v>
       </c>
@@ -2113,8 +2756,11 @@
       <c r="C113" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H113" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="114" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>123</v>
       </c>
@@ -2127,8 +2773,11 @@
       <c r="D114" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H114" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="115" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>124</v>
       </c>
@@ -2138,8 +2787,11 @@
       <c r="C115" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H115" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="116" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>125</v>
       </c>
@@ -2149,8 +2801,11 @@
       <c r="C116" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H116" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="117" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>126</v>
       </c>
@@ -2160,8 +2815,11 @@
       <c r="C117" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="H117" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="118" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>127</v>
       </c>
@@ -2171,53 +2829,74 @@
       <c r="C118" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="G118" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="H118" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="I118" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="J118" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="K118" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="L118" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="M118" s="1" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="119" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B119">
         <v>118</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B120">
         <v>119</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B121">
         <v>120</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B122">
         <v>121</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B123">
         <v>122</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B124">
         <v>123</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B125">
         <v>124</v>
       </c>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B126">
         <v>125</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B127">
         <v>126</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B128">
         <v>127</v>
       </c>
@@ -2673,7 +3352,8 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1" xr:uid="{F7E558BA-FFD6-48B0-805B-6B97F54719C5}"/>
+  <autoFilter ref="A1:M1" xr:uid="{F7E558BA-FFD6-48B0-805B-6B97F54719C5}"/>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>